<commit_message>
seems to work with multiple csources and improves error!
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
+++ b/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Best_Individuals" sheetId="1" r:id="rId1"/>
     <sheet name="Computational_Time" sheetId="2" r:id="rId2"/>
     <sheet name="Final_Errors" sheetId="3" r:id="rId3"/>
+    <sheet name="translational_sector" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
   <si>
     <t>run_id</t>
   </si>
@@ -36,6 +37,9 @@
     <t>ga_error</t>
   </si>
   <si>
+    <t>1.1.1.169</t>
+  </si>
+  <si>
     <t>2.3.3.9</t>
   </si>
   <si>
@@ -48,24 +52,15 @@
     <t>E116</t>
   </si>
   <si>
-    <t>E53</t>
-  </si>
-  <si>
-    <t>2.6.1.55</t>
-  </si>
-  <si>
-    <t>2.8.3.9</t>
-  </si>
-  <si>
-    <t>3.1.3.5</t>
-  </si>
-  <si>
-    <t>3.1.3.97</t>
+    <t>3.5.4.4</t>
   </si>
   <si>
     <t>f</t>
   </si>
   <si>
+    <t>AKGDH</t>
+  </si>
+  <si>
     <t>FUM</t>
   </si>
   <si>
@@ -78,19 +73,7 @@
     <t>CYTBD</t>
   </si>
   <si>
-    <t>O2t</t>
-  </si>
-  <si>
-    <t>PYK</t>
-  </si>
-  <si>
-    <t>ENO</t>
-  </si>
-  <si>
-    <t>PGK</t>
-  </si>
-  <si>
-    <t>GAPD</t>
+    <t>ACKr</t>
   </si>
   <si>
     <t>time_s</t>
@@ -100,6 +83,30 @@
   </si>
   <si>
     <t>r_squared</t>
+  </si>
+  <si>
+    <t>substrate_uptake_id</t>
+  </si>
+  <si>
+    <t>slope</t>
+  </si>
+  <si>
+    <t>intercept</t>
+  </si>
+  <si>
+    <t>EX_glc__D_e</t>
+  </si>
+  <si>
+    <t>EX_ac_e</t>
+  </si>
+  <si>
+    <t>EX_pyr_e</t>
+  </si>
+  <si>
+    <t>EX_succ_e</t>
+  </si>
+  <si>
+    <t>EX_fru_e</t>
   </si>
 </sst>
 </file>
@@ -488,16 +495,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E2">
-        <v>1.890700000000001</v>
+        <v>1.525747498932767</v>
       </c>
       <c r="F2">
-        <v>-0.1615284136897097</v>
+        <v>0.4637931019440965</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -508,16 +515,16 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E3">
-        <v>35.75216181727321</v>
+        <v>1.525830288066733</v>
       </c>
       <c r="F3">
-        <v>-0.1615284136897097</v>
+        <v>0.4637931019440965</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -528,16 +535,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
       <c r="E4">
-        <v>2.2368</v>
+        <v>4.887799999999999</v>
       </c>
       <c r="F4">
-        <v>-0.1615284136897097</v>
+        <v>0.4637931019440965</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -548,16 +555,16 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>101.2734661327629</v>
+        <v>10.50920254045374</v>
       </c>
       <c r="F5">
-        <v>-0.1615284136897097</v>
+        <v>0.4637931019440965</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -568,16 +575,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E6">
         <v>11</v>
       </c>
       <c r="F6">
-        <v>-0.1615284136897097</v>
+        <v>0.4637931019440965</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -585,19 +592,19 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>5.4257</v>
+        <v>1.525747498932767</v>
       </c>
       <c r="F7">
-        <v>-0.04171977966161301</v>
+        <v>0.479243932276341</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -605,19 +612,19 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E8">
-        <v>141.9997487578497</v>
+        <v>1.525830288066733</v>
       </c>
       <c r="F8">
-        <v>-0.04171977966161301</v>
+        <v>0.479243932276341</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -625,19 +632,19 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>75.09260000000002</v>
+        <v>0.9870999999999999</v>
       </c>
       <c r="F9">
-        <v>-0.04171977966161301</v>
+        <v>0.479243932276341</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -645,19 +652,19 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
         <v>15</v>
       </c>
-      <c r="D10" t="s">
-        <v>24</v>
-      </c>
       <c r="E10">
-        <v>172.918919414449</v>
+        <v>4.887799999999999</v>
       </c>
       <c r="F10">
-        <v>-0.04171977966161301</v>
+        <v>0.479243932276341</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -668,16 +675,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E11">
-        <v>11</v>
+        <v>42.30194366912409</v>
       </c>
       <c r="F11">
-        <v>-0.04171977966161301</v>
+        <v>0.479243932276341</v>
       </c>
     </row>
   </sheetData>
@@ -695,10 +702,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -706,10 +713,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>78.37976838300165</v>
+        <v>79.62068387900217</v>
       </c>
       <c r="C2">
-        <v>0.02177215788416713</v>
+        <v>0.02211685663305616</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -717,10 +724,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>72.11052742399988</v>
+        <v>72.52386830199976</v>
       </c>
       <c r="C3">
-        <v>0.02003070206222219</v>
+        <v>0.02014551897277771</v>
       </c>
     </row>
   </sheetData>
@@ -738,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -746,7 +753,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>-0.9531787249165961</v>
+        <v>0.4637931054147842</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -754,7 +761,83 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-0.767089468287973</v>
+        <v>0.4792439374364224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2">
+        <v>-0.002944</v>
+      </c>
+      <c r="C2">
+        <v>0.04992</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3">
+        <v>0.0006351374231102513</v>
+      </c>
+      <c r="C3">
+        <v>0.08555911346944178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <v>-0.004340256958025938</v>
+      </c>
+      <c r="C4">
+        <v>0.04613664490966111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5">
+        <v>-0.004340256958025938</v>
+      </c>
+      <c r="C5">
+        <v>0.04613664490966111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <v>-0.004340256958025938</v>
+      </c>
+      <c r="C6">
+        <v>0.04613664490966111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added convergence rule to prevent unnecessary runtime
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
+++ b/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="40">
   <si>
     <t>run_id</t>
   </si>
@@ -52,9 +52,24 @@
     <t>E116</t>
   </si>
   <si>
+    <t>2.5.1.18</t>
+  </si>
+  <si>
     <t>3.5.4.4</t>
   </si>
   <si>
+    <t>4.1.1.20</t>
+  </si>
+  <si>
+    <t>3.1.3.-</t>
+  </si>
+  <si>
+    <t>E53</t>
+  </si>
+  <si>
+    <t>3.1.3.97</t>
+  </si>
+  <si>
     <t>f</t>
   </si>
   <si>
@@ -73,7 +88,22 @@
     <t>CYTBD</t>
   </si>
   <si>
+    <t>ACONTb</t>
+  </si>
+  <si>
     <t>ACKr</t>
+  </si>
+  <si>
+    <t>NADTRHD</t>
+  </si>
+  <si>
+    <t>PGL</t>
+  </si>
+  <si>
+    <t>O2t</t>
+  </si>
+  <si>
+    <t>GAPD</t>
   </si>
   <si>
     <t>time_s</t>
@@ -464,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -495,16 +525,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2">
-        <v>1.525747498932767</v>
+        <v>6.444866698162853</v>
       </c>
       <c r="F2">
-        <v>0.4637931019440965</v>
+        <v>0.5446667012366359</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -515,16 +545,16 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E3">
-        <v>1.525830288066733</v>
+        <v>0.730256744290638</v>
       </c>
       <c r="F3">
-        <v>0.4637931019440965</v>
+        <v>0.5446667012366359</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -535,16 +565,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E4">
-        <v>4.887799999999999</v>
+        <v>98.1267606119626</v>
       </c>
       <c r="F4">
-        <v>0.4637931019440965</v>
+        <v>0.5446667012366359</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -555,16 +585,16 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E5">
-        <v>10.50920254045374</v>
+        <v>3.402533312260874</v>
       </c>
       <c r="F5">
-        <v>0.4637931019440965</v>
+        <v>0.5446667012366359</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -575,16 +605,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>21.2192669827845</v>
       </c>
       <c r="F6">
-        <v>0.4637931019440965</v>
+        <v>0.5446667012366359</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -592,19 +622,19 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E7">
-        <v>1.525747498932767</v>
+        <v>0.730256744290638</v>
       </c>
       <c r="F7">
-        <v>0.479243932276341</v>
+        <v>0.548603873674456</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -612,19 +642,19 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>1.525830288066733</v>
+        <v>142.2076362442406</v>
       </c>
       <c r="F8">
-        <v>0.479243932276341</v>
+        <v>0.548603873674456</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -632,19 +662,19 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E9">
-        <v>0.9870999999999999</v>
+        <v>0.7078185029471413</v>
       </c>
       <c r="F9">
-        <v>0.479243932276341</v>
+        <v>0.548603873674456</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -652,19 +682,19 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E10">
-        <v>4.887799999999999</v>
+        <v>11.23623998234263</v>
       </c>
       <c r="F10">
-        <v>0.479243932276341</v>
+        <v>0.548603873674456</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -672,19 +702,819 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11">
+        <v>3.534145152442551</v>
+      </c>
+      <c r="F11">
+        <v>0.548603873674456</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12">
+        <v>6.444866698162853</v>
+      </c>
+      <c r="F12">
+        <v>0.5488237483404947</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13">
+        <v>0.730256744290638</v>
+      </c>
+      <c r="F13">
+        <v>0.5488237483404947</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14">
+        <v>1588.789338843621</v>
+      </c>
+      <c r="F14">
+        <v>0.5488237483404947</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>2.396756763579956</v>
+      </c>
+      <c r="F15">
+        <v>0.5488237483404947</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16">
+        <v>3.53414515244255</v>
+      </c>
+      <c r="F16">
+        <v>0.5488237483404947</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17">
+        <v>6.444866698162853</v>
+      </c>
+      <c r="F17">
+        <v>0.5506706007700732</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18">
+        <v>0.730256744290638</v>
+      </c>
+      <c r="F18">
+        <v>0.5506706007700732</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19">
+        <v>1166.229269813276</v>
+      </c>
+      <c r="F19">
+        <v>0.5506706007700732</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20">
+        <v>25.93490304216703</v>
+      </c>
+      <c r="F20">
+        <v>0.5506706007700732</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21">
+        <v>3.53414515244255</v>
+      </c>
+      <c r="F21">
+        <v>0.5506706007700732</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22">
+        <v>5</v>
+      </c>
+      <c r="B22" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F22">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <v>5</v>
+      </c>
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F23">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24">
+        <v>3.466969363495611</v>
+      </c>
+      <c r="F24">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
         <v>10</v>
       </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11">
-        <v>42.30194366912409</v>
-      </c>
-      <c r="F11">
-        <v>0.479243932276341</v>
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25">
+        <v>21.58888177380997</v>
+      </c>
+      <c r="F25">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26">
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26">
+        <v>6.977420574924071</v>
+      </c>
+      <c r="F26">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F27">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F28">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29">
+        <v>3.466969363495612</v>
+      </c>
+      <c r="F29">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30">
+        <v>21.58888177380997</v>
+      </c>
+      <c r="F30">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31">
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31">
+        <v>6.977420574924071</v>
+      </c>
+      <c r="F31">
+        <v>0.5551771850719225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32">
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F32">
+        <v>0.5553281975809238</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F33">
+        <v>0.5553281975809238</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34">
+        <v>3.466969363495612</v>
+      </c>
+      <c r="F34">
+        <v>0.5553281975809238</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" t="s">
+        <v>22</v>
+      </c>
+      <c r="E35">
+        <v>139.5030938626211</v>
+      </c>
+      <c r="F35">
+        <v>0.5553281975809238</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E36">
+        <v>4.552456757832201</v>
+      </c>
+      <c r="F36">
+        <v>0.5553281975809238</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37">
+        <v>8</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F37">
+        <v>0.556958190187514</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38">
+        <v>8</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" t="s">
+        <v>26</v>
+      </c>
+      <c r="E38">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F38">
+        <v>0.556958190187514</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39">
+        <v>8</v>
+      </c>
+      <c r="B39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39">
+        <v>19.11995689233207</v>
+      </c>
+      <c r="F39">
+        <v>0.556958190187514</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40">
+        <v>8</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" t="s">
+        <v>21</v>
+      </c>
+      <c r="E40">
+        <v>3.466969363495612</v>
+      </c>
+      <c r="F40">
+        <v>0.556958190187514</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41">
+        <v>8</v>
+      </c>
+      <c r="B41" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E41">
+        <v>4.552456757832201</v>
+      </c>
+      <c r="F41">
+        <v>0.556958190187514</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" t="s">
+        <v>19</v>
+      </c>
+      <c r="E42">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F42">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" t="s">
+        <v>26</v>
+      </c>
+      <c r="E43">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F43">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44">
+        <v>9</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" t="s">
+        <v>28</v>
+      </c>
+      <c r="E44">
+        <v>18.5511243541397</v>
+      </c>
+      <c r="F44">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45">
+        <v>9</v>
+      </c>
+      <c r="B45" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" t="s">
+        <v>21</v>
+      </c>
+      <c r="E45">
+        <v>3.466969363495612</v>
+      </c>
+      <c r="F45">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46">
+        <v>9</v>
+      </c>
+      <c r="B46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46">
+        <v>4.552456757832201</v>
+      </c>
+      <c r="F46">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47">
+        <v>10</v>
+      </c>
+      <c r="B47" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" t="s">
+        <v>19</v>
+      </c>
+      <c r="E47">
+        <v>0.6433776556481242</v>
+      </c>
+      <c r="F47">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48">
+        <v>10</v>
+      </c>
+      <c r="B48" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" t="s">
+        <v>26</v>
+      </c>
+      <c r="E48">
+        <v>2.128998792076188</v>
+      </c>
+      <c r="F48">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49">
+        <v>10</v>
+      </c>
+      <c r="B49" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" t="s">
+        <v>17</v>
+      </c>
+      <c r="D49" t="s">
+        <v>28</v>
+      </c>
+      <c r="E49">
+        <v>18.5511243541397</v>
+      </c>
+      <c r="F49">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50">
+        <v>10</v>
+      </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" t="s">
+        <v>21</v>
+      </c>
+      <c r="E50">
+        <v>3.466969363495612</v>
+      </c>
+      <c r="F50">
+        <v>0.5569802581793465</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51">
+        <v>10</v>
+      </c>
+      <c r="B51" t="s">
+        <v>15</v>
+      </c>
+      <c r="C51" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51" t="s">
+        <v>27</v>
+      </c>
+      <c r="E51">
+        <v>4.552456757832201</v>
+      </c>
+      <c r="F51">
+        <v>0.5569802581793465</v>
       </c>
     </row>
   </sheetData>
@@ -694,7 +1524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -702,10 +1532,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -713,10 +1543,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>79.62068387900217</v>
+        <v>524.8897478779982</v>
       </c>
       <c r="C2">
-        <v>0.02211685663305616</v>
+        <v>0.1458027077438884</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -724,10 +1554,98 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>72.52386830199976</v>
+        <v>547.2470398800069</v>
       </c>
       <c r="C3">
-        <v>0.02014551897277771</v>
+        <v>0.1520130666333352</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>533.910228534005</v>
+      </c>
+      <c r="C4">
+        <v>0.1483083968150014</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>531.7993736609933</v>
+      </c>
+      <c r="C5">
+        <v>0.1477220482391648</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>540.7080137489975</v>
+      </c>
+      <c r="C6">
+        <v>0.1501966704858326</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>504.6100911490066</v>
+      </c>
+      <c r="C7">
+        <v>0.1401694697636129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>532.0943992130051</v>
+      </c>
+      <c r="C8">
+        <v>0.1478039997813903</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>557.0111524749955</v>
+      </c>
+      <c r="C9">
+        <v>0.1547253201319432</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>578.2347192809975</v>
+      </c>
+      <c r="C10">
+        <v>0.1606207553558326</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>489.6022432530008</v>
+      </c>
+      <c r="C11">
+        <v>0.1360006231258336</v>
       </c>
     </row>
   </sheetData>
@@ -737,7 +1655,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -745,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -753,7 +1671,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.4637931054147842</v>
+        <v>0.5446667038958003</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -761,7 +1679,71 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.4792439374364224</v>
+        <v>0.5486038764172775</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0.5488237511105045</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0.5506706035391147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>0.5551771892155042</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0.5551771892155042</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0.5553282019168432</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0.5569581946713972</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0.5569802626671422</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0.5569802626671422</v>
       </c>
     </row>
   </sheetData>
@@ -776,18 +1758,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B2">
         <v>-0.002944</v>
@@ -798,7 +1780,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>0.0006351374231102513</v>
@@ -809,7 +1791,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B4">
         <v>-0.004340256958025938</v>
@@ -820,7 +1802,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>-0.004340256958025938</v>
@@ -831,7 +1813,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B6">
         <v>-0.004340256958025938</v>

</xml_diff>

<commit_message>
seems to work for uniprot parsing as well
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
+++ b/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="35">
   <si>
     <t>run_id</t>
   </si>
@@ -37,73 +37,58 @@
     <t>ga_error</t>
   </si>
   <si>
-    <t>1.1.1.169</t>
-  </si>
-  <si>
-    <t>2.3.3.9</t>
-  </si>
-  <si>
-    <t>4.1.3.42</t>
-  </si>
-  <si>
-    <t>4.2.1.17</t>
-  </si>
-  <si>
-    <t>E116</t>
-  </si>
-  <si>
-    <t>2.5.1.18</t>
-  </si>
-  <si>
-    <t>3.5.4.4</t>
-  </si>
-  <si>
-    <t>4.1.1.20</t>
-  </si>
-  <si>
-    <t>3.1.3.-</t>
-  </si>
-  <si>
-    <t>E53</t>
-  </si>
-  <si>
-    <t>3.1.3.97</t>
+    <t>P00864</t>
+  </si>
+  <si>
+    <t>P0A6P9</t>
+  </si>
+  <si>
+    <t>P0AB71</t>
+  </si>
+  <si>
+    <t>P25516</t>
+  </si>
+  <si>
+    <t>P52697</t>
+  </si>
+  <si>
+    <t>P0A991</t>
+  </si>
+  <si>
+    <t>P36683</t>
   </si>
   <si>
     <t>f</t>
   </si>
   <si>
-    <t>AKGDH</t>
-  </si>
-  <si>
-    <t>FUM</t>
-  </si>
-  <si>
-    <t>PTAr</t>
-  </si>
-  <si>
-    <t>MDH</t>
-  </si>
-  <si>
-    <t>CYTBD</t>
-  </si>
-  <si>
-    <t>ACONTb</t>
-  </si>
-  <si>
-    <t>ACKr</t>
-  </si>
-  <si>
-    <t>NADTRHD</t>
-  </si>
-  <si>
-    <t>PGL</t>
-  </si>
-  <si>
-    <t>O2t</t>
-  </si>
-  <si>
-    <t>GAPD</t>
+    <t>b</t>
+  </si>
+  <si>
+    <t>CE_PPC_P00864</t>
+  </si>
+  <si>
+    <t>CE_ENO_P0A6P9</t>
+  </si>
+  <si>
+    <t>CE_FBA_P0AB71</t>
+  </si>
+  <si>
+    <t>CE_ACONTb_P25516</t>
+  </si>
+  <si>
+    <t>CE_PGL_P52697</t>
+  </si>
+  <si>
+    <t>CE_FBA_P0A991</t>
+  </si>
+  <si>
+    <t>CE_ACONTa_P25516</t>
+  </si>
+  <si>
+    <t>CE_ACONTb_P36683</t>
+  </si>
+  <si>
+    <t>CE_ACONTa_P36683</t>
   </si>
   <si>
     <t>time_s</t>
@@ -494,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -525,16 +510,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>6.444866698162853</v>
+        <v>4.635200000000001</v>
       </c>
       <c r="F2">
-        <v>0.5446667012366359</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -542,19 +527,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E3">
-        <v>0.730256744290638</v>
+        <v>4.635200000000001</v>
       </c>
       <c r="F3">
-        <v>0.5446667012366359</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -562,19 +547,19 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E4">
-        <v>98.1267606119626</v>
+        <v>5.531455848447435</v>
       </c>
       <c r="F4">
-        <v>0.5446667012366359</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -582,19 +567,19 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>3.402533312260874</v>
+        <v>7.554538260569988</v>
       </c>
       <c r="F5">
-        <v>0.5446667012366359</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -602,919 +587,599 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
       <c r="E6">
-        <v>21.2192669827845</v>
+        <v>0.9620446221468493</v>
       </c>
       <c r="F6">
-        <v>0.5446667012366359</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
       <c r="E7">
-        <v>0.730256744290638</v>
+        <v>1.5402</v>
       </c>
       <c r="F7">
-        <v>0.548603873674456</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E8">
-        <v>142.2076362442406</v>
+        <v>1.633690514792494</v>
       </c>
       <c r="F8">
-        <v>0.548603873674456</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>0.7078185029471413</v>
+        <v>33.92535044172813</v>
       </c>
       <c r="F9">
-        <v>0.548603873674456</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
         <v>13</v>
       </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E10">
-        <v>11.23623998234263</v>
+        <v>3.281799999999999</v>
       </c>
       <c r="F10">
-        <v>0.548603873674456</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E11">
-        <v>3.534145152442551</v>
+        <v>1.890999163089456</v>
       </c>
       <c r="F11">
-        <v>0.548603873674456</v>
+        <v>0.2932605219734812</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E12">
-        <v>6.444866698162853</v>
+        <v>4.04709763232365</v>
       </c>
       <c r="F12">
-        <v>0.5488237483404947</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E13">
-        <v>0.730256744290638</v>
+        <v>1.2496</v>
       </c>
       <c r="F13">
-        <v>0.5488237483404947</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E14">
-        <v>1588.789338843621</v>
+        <v>0.5326465724254145</v>
       </c>
       <c r="F14">
-        <v>0.5488237483404947</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
         <v>17</v>
       </c>
-      <c r="D15" t="s">
-        <v>24</v>
-      </c>
       <c r="E15">
-        <v>2.396756763579956</v>
+        <v>0.4556573814670354</v>
       </c>
       <c r="F15">
-        <v>0.5488237483404947</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
       </c>
       <c r="E16">
-        <v>3.53414515244255</v>
+        <v>961.842150660532</v>
       </c>
       <c r="F16">
-        <v>0.5488237483404947</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E17">
-        <v>6.444866698162853</v>
+        <v>5.8129</v>
       </c>
       <c r="F17">
-        <v>0.5506706007700732</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E18">
-        <v>0.730256744290638</v>
+        <v>5.689534798269007</v>
       </c>
       <c r="F18">
-        <v>0.5506706007700732</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E19">
-        <v>1166.229269813276</v>
+        <v>2.430939310141345</v>
       </c>
       <c r="F19">
-        <v>0.5506706007700732</v>
+        <v>0.2992442350300034</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E20">
-        <v>25.93490304216703</v>
+        <v>3.988527426449629</v>
       </c>
       <c r="F20">
-        <v>0.5506706007700732</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E21">
-        <v>3.53414515244255</v>
+        <v>0.5326465724254145</v>
       </c>
       <c r="F21">
-        <v>0.5506706007700732</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
         <v>17</v>
       </c>
-      <c r="D22" t="s">
-        <v>19</v>
-      </c>
       <c r="E22">
-        <v>0.6433776556481242</v>
+        <v>0.444772934192277</v>
       </c>
       <c r="F22">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E23">
-        <v>2.128998792076188</v>
+        <v>82.13675452663207</v>
       </c>
       <c r="F23">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E24">
-        <v>3.466969363495611</v>
+        <v>6.724353018628222</v>
       </c>
       <c r="F24">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D25" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E25">
-        <v>21.58888177380997</v>
+        <v>5.075656237250306</v>
       </c>
       <c r="F25">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C26" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E26">
-        <v>6.977420574924071</v>
+        <v>3.988527426449629</v>
       </c>
       <c r="F26">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E27">
-        <v>0.6433776556481242</v>
+        <v>0.5326465724254145</v>
       </c>
       <c r="F27">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" t="s">
         <v>17</v>
       </c>
-      <c r="D28" t="s">
-        <v>26</v>
-      </c>
       <c r="E28">
-        <v>2.128998792076188</v>
+        <v>0.2659337772268022</v>
       </c>
       <c r="F28">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E29">
-        <v>3.466969363495612</v>
+        <v>51.12432174134177</v>
       </c>
       <c r="F29">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E30">
-        <v>21.58888177380997</v>
+        <v>5.075656237250307</v>
       </c>
       <c r="F30">
-        <v>0.5551771850719225</v>
+        <v>0.2992563521321562</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D31" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>6.977420574924071</v>
+        <v>3.756476057634403</v>
       </c>
       <c r="F31">
-        <v>0.5551771850719225</v>
+        <v>0.2992565162214604</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E32">
-        <v>0.6433776556481242</v>
+        <v>0.5488096236806524</v>
       </c>
       <c r="F32">
-        <v>0.5553281975809238</v>
+        <v>0.2992565162214604</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C33" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" t="s">
         <v>17</v>
       </c>
-      <c r="D33" t="s">
-        <v>26</v>
-      </c>
       <c r="E33">
-        <v>2.128998792076188</v>
+        <v>0.2207387562692917</v>
       </c>
       <c r="F33">
-        <v>0.5553281975809238</v>
+        <v>0.2992565162214604</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E34">
-        <v>3.466969363495612</v>
+        <v>30.57904264687695</v>
       </c>
       <c r="F34">
-        <v>0.5553281975809238</v>
+        <v>0.2992565162214604</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E35">
-        <v>139.5030938626211</v>
+        <v>10.69660415355141</v>
       </c>
       <c r="F35">
-        <v>0.5553281975809238</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E36">
-        <v>4.552456757832201</v>
-      </c>
-      <c r="F36">
-        <v>0.5553281975809238</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37">
-        <v>8</v>
-      </c>
-      <c r="B37" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" t="s">
-        <v>17</v>
-      </c>
-      <c r="D37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37">
-        <v>0.6433776556481242</v>
-      </c>
-      <c r="F37">
-        <v>0.556958190187514</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38">
-        <v>8</v>
-      </c>
-      <c r="B38" t="s">
-        <v>14</v>
-      </c>
-      <c r="C38" t="s">
-        <v>17</v>
-      </c>
-      <c r="D38" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38">
-        <v>2.128998792076188</v>
-      </c>
-      <c r="F38">
-        <v>0.556958190187514</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39">
-        <v>8</v>
-      </c>
-      <c r="B39" t="s">
-        <v>13</v>
-      </c>
-      <c r="C39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" t="s">
-        <v>25</v>
-      </c>
-      <c r="E39">
-        <v>19.11995689233207</v>
-      </c>
-      <c r="F39">
-        <v>0.556958190187514</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40">
-        <v>8</v>
-      </c>
-      <c r="B40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" t="s">
-        <v>17</v>
-      </c>
-      <c r="D40" t="s">
-        <v>21</v>
-      </c>
-      <c r="E40">
-        <v>3.466969363495612</v>
-      </c>
-      <c r="F40">
-        <v>0.556958190187514</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41">
-        <v>8</v>
-      </c>
-      <c r="B41" t="s">
-        <v>15</v>
-      </c>
-      <c r="C41" t="s">
-        <v>17</v>
-      </c>
-      <c r="D41" t="s">
-        <v>27</v>
-      </c>
-      <c r="E41">
-        <v>4.552456757832201</v>
-      </c>
-      <c r="F41">
-        <v>0.556958190187514</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42">
-        <v>9</v>
-      </c>
-      <c r="B42" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42">
-        <v>0.6433776556481242</v>
-      </c>
-      <c r="F42">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43">
-        <v>9</v>
-      </c>
-      <c r="B43" t="s">
-        <v>14</v>
-      </c>
-      <c r="C43" t="s">
-        <v>17</v>
-      </c>
-      <c r="D43" t="s">
-        <v>26</v>
-      </c>
-      <c r="E43">
-        <v>2.128998792076188</v>
-      </c>
-      <c r="F43">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44">
-        <v>9</v>
-      </c>
-      <c r="B44" t="s">
-        <v>16</v>
-      </c>
-      <c r="C44" t="s">
-        <v>17</v>
-      </c>
-      <c r="D44" t="s">
-        <v>28</v>
-      </c>
-      <c r="E44">
-        <v>18.5511243541397</v>
-      </c>
-      <c r="F44">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45">
-        <v>9</v>
-      </c>
-      <c r="B45" t="s">
-        <v>9</v>
-      </c>
-      <c r="C45" t="s">
-        <v>17</v>
-      </c>
-      <c r="D45" t="s">
-        <v>21</v>
-      </c>
-      <c r="E45">
-        <v>3.466969363495612</v>
-      </c>
-      <c r="F45">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46">
-        <v>9</v>
-      </c>
-      <c r="B46" t="s">
-        <v>15</v>
-      </c>
-      <c r="C46" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" t="s">
-        <v>27</v>
-      </c>
-      <c r="E46">
-        <v>4.552456757832201</v>
-      </c>
-      <c r="F46">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47">
-        <v>10</v>
-      </c>
-      <c r="B47" t="s">
-        <v>7</v>
-      </c>
-      <c r="C47" t="s">
-        <v>17</v>
-      </c>
-      <c r="D47" t="s">
-        <v>19</v>
-      </c>
-      <c r="E47">
-        <v>0.6433776556481242</v>
-      </c>
-      <c r="F47">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48">
-        <v>10</v>
-      </c>
-      <c r="B48" t="s">
-        <v>14</v>
-      </c>
-      <c r="C48" t="s">
-        <v>17</v>
-      </c>
-      <c r="D48" t="s">
-        <v>26</v>
-      </c>
-      <c r="E48">
-        <v>2.128998792076188</v>
-      </c>
-      <c r="F48">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49">
-        <v>10</v>
-      </c>
-      <c r="B49" t="s">
-        <v>16</v>
-      </c>
-      <c r="C49" t="s">
-        <v>17</v>
-      </c>
-      <c r="D49" t="s">
-        <v>28</v>
-      </c>
-      <c r="E49">
-        <v>18.5511243541397</v>
-      </c>
-      <c r="F49">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
-      <c r="A50">
-        <v>10</v>
-      </c>
-      <c r="B50" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50" t="s">
-        <v>17</v>
-      </c>
-      <c r="D50" t="s">
-        <v>21</v>
-      </c>
-      <c r="E50">
-        <v>3.466969363495612</v>
-      </c>
-      <c r="F50">
-        <v>0.5569802581793465</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
-      <c r="A51">
-        <v>10</v>
-      </c>
-      <c r="B51" t="s">
-        <v>15</v>
-      </c>
-      <c r="C51" t="s">
-        <v>17</v>
-      </c>
-      <c r="D51" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51">
-        <v>4.552456757832201</v>
-      </c>
-      <c r="F51">
-        <v>0.5569802581793465</v>
+        <v>0.2992565162214604</v>
       </c>
     </row>
   </sheetData>
@@ -1524,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1532,10 +1197,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1543,10 +1208,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>524.8897478779982</v>
+        <v>652.1993414109966</v>
       </c>
       <c r="C2">
-        <v>0.1458027077438884</v>
+        <v>0.1811664837252768</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1554,10 +1219,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>547.2470398800069</v>
+        <v>624.6746508350006</v>
       </c>
       <c r="C3">
-        <v>0.1520130666333352</v>
+        <v>0.1735207363430557</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1565,10 +1230,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>533.910228534005</v>
+        <v>630.1063828060032</v>
       </c>
       <c r="C4">
-        <v>0.1483083968150014</v>
+        <v>0.1750295507794453</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1576,10 +1241,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>531.7993736609933</v>
+        <v>640.7010529990002</v>
       </c>
       <c r="C5">
-        <v>0.1477220482391648</v>
+        <v>0.1779725147219445</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1587,65 +1252,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>540.7080137489975</v>
+        <v>628.2668139600028</v>
       </c>
       <c r="C6">
-        <v>0.1501966704858326</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>504.6100911490066</v>
-      </c>
-      <c r="C7">
-        <v>0.1401694697636129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>532.0943992130051</v>
-      </c>
-      <c r="C8">
-        <v>0.1478039997813903</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>557.0111524749955</v>
-      </c>
-      <c r="C9">
-        <v>0.1547253201319432</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>578.2347192809975</v>
-      </c>
-      <c r="C10">
-        <v>0.1606207553558326</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>489.6022432530008</v>
-      </c>
-      <c r="C11">
-        <v>0.1360006231258336</v>
+        <v>0.1745185594333341</v>
       </c>
     </row>
   </sheetData>
@@ -1655,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1663,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1671,7 +1281,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.5446667038958003</v>
+        <v>0.2932606537898456</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1679,7 +1289,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.5486038764172775</v>
+        <v>0.2992443668463679</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1687,7 +1297,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.5488237511105045</v>
+        <v>0.2992564839485203</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1695,7 +1305,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.5506706035391147</v>
+        <v>0.2992564839485203</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1703,47 +1313,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.5551771892155042</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>0.5551771892155042</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>0.5553282019168432</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0.5569581946713972</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>0.5569802626671422</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>0.5569802626671422</v>
+        <v>0.2992566480378244</v>
       </c>
     </row>
   </sheetData>
@@ -1758,18 +1328,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B2">
         <v>-0.002944</v>
@@ -1780,18 +1350,18 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B3">
-        <v>0.0006351374231102513</v>
+        <v>-0.004340256958025938</v>
       </c>
       <c r="C3">
-        <v>0.08555911346944178</v>
+        <v>0.04613664490966111</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B4">
         <v>-0.004340256958025938</v>
@@ -1802,7 +1372,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B5">
         <v>-0.004340256958025938</v>
@@ -1813,7 +1383,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B6">
         <v>-0.004340256958025938</v>

</xml_diff>

<commit_message>
updated the framework for getting out of local minima
</commit_message>
<xml_diff>
--- a/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
+++ b/Results/pam_parametrizer_diagnostics_ecolicore_false_multiple_csources2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="53">
   <si>
     <t>run_id</t>
   </si>
@@ -58,6 +58,33 @@
     <t>P36683</t>
   </si>
   <si>
+    <t>P06959_P0A9P0_P0AFG8</t>
+  </si>
+  <si>
+    <t>P09832_P09831</t>
+  </si>
+  <si>
+    <t>P23538</t>
+  </si>
+  <si>
+    <t>P39451</t>
+  </si>
+  <si>
+    <t>P0A9N4_P09373</t>
+  </si>
+  <si>
+    <t>P0AC53</t>
+  </si>
+  <si>
+    <t>P0AGE9_P0A836</t>
+  </si>
+  <si>
+    <t>P32674_P32675</t>
+  </si>
+  <si>
+    <t>P37689</t>
+  </si>
+  <si>
     <t>f</t>
   </si>
   <si>
@@ -89,6 +116,33 @@
   </si>
   <si>
     <t>CE_ACONTa_P36683</t>
+  </si>
+  <si>
+    <t>CE_PDH_P06959_P0A9P0_P0AFG8</t>
+  </si>
+  <si>
+    <t>CE_GLUSy_P09832_P09831</t>
+  </si>
+  <si>
+    <t>CE_PPS_P23538</t>
+  </si>
+  <si>
+    <t>CE_ALCD2x_P39451</t>
+  </si>
+  <si>
+    <t>CE_PFL_P0A9N4_P09373</t>
+  </si>
+  <si>
+    <t>CE_G6PDH2r_P0AC53</t>
+  </si>
+  <si>
+    <t>CE_SUCOAS_P0AGE9_P0A836</t>
+  </si>
+  <si>
+    <t>CE_PFL_P32674_P32675</t>
+  </si>
+  <si>
+    <t>CE_PGM_P37689</t>
   </si>
   <si>
     <t>time_s</t>
@@ -479,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -510,16 +564,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>4.635200000000001</v>
       </c>
       <c r="F2">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -530,16 +584,16 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E3">
         <v>4.635200000000001</v>
       </c>
       <c r="F3">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -550,16 +604,16 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E4">
-        <v>5.531455848447435</v>
+        <v>28.59274883824098</v>
       </c>
       <c r="F4">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -570,16 +624,16 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E5">
-        <v>7.554538260569988</v>
+        <v>15.85414291411859</v>
       </c>
       <c r="F5">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -590,16 +644,16 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E6">
-        <v>0.9620446221468493</v>
+        <v>0.807140523706377</v>
       </c>
       <c r="F6">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -610,16 +664,16 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E7">
-        <v>1.5402</v>
+        <v>1.735971618668857</v>
       </c>
       <c r="F7">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -630,16 +684,16 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>1.633690514792494</v>
+        <v>3.87899353555691</v>
       </c>
       <c r="F8">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -650,16 +704,16 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E9">
-        <v>33.92535044172813</v>
+        <v>2.405676721895346</v>
       </c>
       <c r="F9">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -670,16 +724,16 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E10">
-        <v>3.281799999999999</v>
+        <v>1.911299920628384</v>
       </c>
       <c r="F10">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -690,16 +744,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E11">
-        <v>1.890999163089456</v>
+        <v>1.803854826119102</v>
       </c>
       <c r="F11">
-        <v>0.2932605219734812</v>
+        <v>0.4934548843418713</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -707,19 +761,19 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E12">
-        <v>4.04709763232365</v>
+        <v>0.7618868965110764</v>
       </c>
       <c r="F12">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -730,16 +784,16 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E13">
-        <v>1.2496</v>
+        <v>0.9931487517841856</v>
       </c>
       <c r="F13">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -747,19 +801,19 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>0.5326465724254145</v>
+        <v>308.2048379741487</v>
       </c>
       <c r="F14">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -767,19 +821,19 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E15">
-        <v>0.4556573814670354</v>
+        <v>28.17067133283505</v>
       </c>
       <c r="F15">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -790,16 +844,16 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E16">
-        <v>961.842150660532</v>
+        <v>4.634194869157138</v>
       </c>
       <c r="F16">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -807,19 +861,19 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E17">
-        <v>5.8129</v>
+        <v>4.4574</v>
       </c>
       <c r="F17">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -830,16 +884,16 @@
         <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E18">
-        <v>5.689534798269007</v>
+        <v>3.032877587749125</v>
       </c>
       <c r="F18">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -847,19 +901,19 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E19">
-        <v>2.430939310141345</v>
+        <v>5.476078872775786</v>
       </c>
       <c r="F19">
-        <v>0.2992442350300034</v>
+        <v>0.5053434010157347</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -867,19 +921,19 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D20" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E20">
-        <v>3.988527426449629</v>
+        <v>3.070627149815392</v>
       </c>
       <c r="F20">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -887,19 +941,19 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E21">
-        <v>0.5326465724254145</v>
+        <v>95.78110364218348</v>
       </c>
       <c r="F21">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -907,19 +961,19 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E22">
-        <v>0.444772934192277</v>
+        <v>11.78547385894701</v>
       </c>
       <c r="F22">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -927,19 +981,19 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E23">
-        <v>82.13675452663207</v>
+        <v>31.89448054664502</v>
       </c>
       <c r="F23">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -950,16 +1004,16 @@
         <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E24">
-        <v>6.724353018628222</v>
+        <v>3.304127718544458</v>
       </c>
       <c r="F24">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -967,19 +1021,19 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E25">
-        <v>5.075656237250306</v>
+        <v>43.18593032344824</v>
       </c>
       <c r="F25">
-        <v>0.2992563521321562</v>
+        <v>0.5054793609644952</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -987,19 +1041,19 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E26">
-        <v>3.988527426449629</v>
+        <v>6.952275870974174</v>
       </c>
       <c r="F26">
-        <v>0.2992563521321562</v>
+        <v>0.5055339172885536</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1007,19 +1061,19 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E27">
-        <v>0.5326465724254145</v>
+        <v>11.9896736668161</v>
       </c>
       <c r="F27">
-        <v>0.2992563521321562</v>
+        <v>0.5055339172885536</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1027,19 +1081,19 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E28">
-        <v>0.2659337772268022</v>
+        <v>1.480338239039642</v>
       </c>
       <c r="F28">
-        <v>0.2992563521321562</v>
+        <v>0.5055339172885536</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1047,19 +1101,19 @@
         <v>4</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E29">
-        <v>51.12432174134177</v>
+        <v>3.611674324445969</v>
       </c>
       <c r="F29">
-        <v>0.2992563521321562</v>
+        <v>0.5055339172885536</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1067,19 +1121,19 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E30">
-        <v>5.075656237250307</v>
+        <v>56.68094281696187</v>
       </c>
       <c r="F30">
-        <v>0.2992563521321562</v>
+        <v>0.5055339172885536</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1087,19 +1141,19 @@
         <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E31">
-        <v>3.756476057634403</v>
+        <v>2.401892166996265</v>
       </c>
       <c r="F31">
-        <v>0.2992565162214604</v>
+        <v>0.5057333370226764</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1107,19 +1161,19 @@
         <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E32">
-        <v>0.5488096236806524</v>
+        <v>3.685096603181675</v>
       </c>
       <c r="F32">
-        <v>0.2992565162214604</v>
+        <v>0.5057333370226764</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1127,19 +1181,19 @@
         <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E33">
-        <v>0.2207387562692917</v>
+        <v>3.670858988662413</v>
       </c>
       <c r="F33">
-        <v>0.2992565162214604</v>
+        <v>0.5057333370226764</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1147,19 +1201,19 @@
         <v>5</v>
       </c>
       <c r="B34" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C34" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E34">
-        <v>30.57904264687695</v>
+        <v>28.76617286094434</v>
       </c>
       <c r="F34">
-        <v>0.2992565162214604</v>
+        <v>0.5057333370226764</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1167,19 +1221,619 @@
         <v>5</v>
       </c>
       <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35">
+        <v>235313.8757478297</v>
+      </c>
+      <c r="F35">
+        <v>0.5057333370226764</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" t="s">
+        <v>22</v>
+      </c>
+      <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36">
+        <v>153.2073870533948</v>
+      </c>
+      <c r="F36">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37">
+        <v>6</v>
+      </c>
+      <c r="B37" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" t="s">
+        <v>22</v>
+      </c>
+      <c r="D37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37">
+        <v>3.59099774552855</v>
+      </c>
+      <c r="F37">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E38">
+        <v>23.71138000690564</v>
+      </c>
+      <c r="F38">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39">
+        <v>6</v>
+      </c>
+      <c r="B39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" t="s">
+        <v>22</v>
+      </c>
+      <c r="D39" t="s">
+        <v>35</v>
+      </c>
+      <c r="E39">
+        <v>3.727402874972166</v>
+      </c>
+      <c r="F39">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40">
+        <v>6</v>
+      </c>
+      <c r="B40" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" t="s">
+        <v>35</v>
+      </c>
+      <c r="E40">
+        <v>3.088413219263043</v>
+      </c>
+      <c r="F40">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41">
+        <v>6</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E41">
+        <v>4.014786135997897</v>
+      </c>
+      <c r="F41">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" t="s">
+        <v>36</v>
+      </c>
+      <c r="E42">
+        <v>16.06538782929406</v>
+      </c>
+      <c r="F42">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43">
+        <v>6</v>
+      </c>
+      <c r="B43" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43">
+        <v>4.67634488031748</v>
+      </c>
+      <c r="F43">
+        <v>0.5057930528525501</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44">
+        <v>7</v>
+      </c>
+      <c r="B44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C44" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44">
+        <v>3.094114476844106</v>
+      </c>
+      <c r="F44">
+        <v>0.5058249270604682</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45">
+        <v>7</v>
+      </c>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="E45">
+        <v>3.924853041651504</v>
+      </c>
+      <c r="F45">
+        <v>0.5058249270604682</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46">
+        <v>7</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46">
+        <v>2.123243726360994</v>
+      </c>
+      <c r="F46">
+        <v>0.5058249270604682</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
         <v>12</v>
       </c>
-      <c r="C35" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" t="s">
-        <v>23</v>
-      </c>
-      <c r="E35">
-        <v>10.69660415355141</v>
-      </c>
-      <c r="F35">
-        <v>0.2992565162214604</v>
+      <c r="C47" t="s">
+        <v>23</v>
+      </c>
+      <c r="D47" t="s">
+        <v>31</v>
+      </c>
+      <c r="E47">
+        <v>15.36913866466479</v>
+      </c>
+      <c r="F47">
+        <v>0.5058249270604682</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
+        <v>23</v>
+      </c>
+      <c r="D48" t="s">
+        <v>28</v>
+      </c>
+      <c r="E48">
+        <v>336145.7479215431</v>
+      </c>
+      <c r="F48">
+        <v>0.5058249270604682</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49">
+        <v>8</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" t="s">
+        <v>22</v>
+      </c>
+      <c r="D49" t="s">
+        <v>37</v>
+      </c>
+      <c r="E49">
+        <v>203.1892831489596</v>
+      </c>
+      <c r="F49">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50">
+        <v>8</v>
+      </c>
+      <c r="B50" t="s">
+        <v>18</v>
+      </c>
+      <c r="C50" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50">
+        <v>4126.071175981778</v>
+      </c>
+      <c r="F50">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51">
+        <v>8</v>
+      </c>
+      <c r="B51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" t="s">
+        <v>23</v>
+      </c>
+      <c r="D51" t="s">
+        <v>38</v>
+      </c>
+      <c r="E51">
+        <v>8.494813737325087</v>
+      </c>
+      <c r="F51">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52">
+        <v>8</v>
+      </c>
+      <c r="B52" t="s">
+        <v>19</v>
+      </c>
+      <c r="C52" t="s">
+        <v>22</v>
+      </c>
+      <c r="D52" t="s">
+        <v>39</v>
+      </c>
+      <c r="E52">
+        <v>108.9598572640456</v>
+      </c>
+      <c r="F52">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53">
+        <v>8</v>
+      </c>
+      <c r="B53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C53" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" t="s">
+        <v>39</v>
+      </c>
+      <c r="E53">
+        <v>162.7725234386829</v>
+      </c>
+      <c r="F53">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54">
+        <v>8</v>
+      </c>
+      <c r="B54" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" t="s">
+        <v>40</v>
+      </c>
+      <c r="E54">
+        <v>7.523963425671091</v>
+      </c>
+      <c r="F54">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55">
+        <v>8</v>
+      </c>
+      <c r="B55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55" t="s">
+        <v>41</v>
+      </c>
+      <c r="E55">
+        <v>90.06898243221158</v>
+      </c>
+      <c r="F55">
+        <v>0.5073603500357441</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56">
+        <v>9</v>
+      </c>
+      <c r="B56" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" t="s">
+        <v>29</v>
+      </c>
+      <c r="E56">
+        <v>1.929517162476951</v>
+      </c>
+      <c r="F56">
+        <v>0.5075966032810001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57">
+        <v>9</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" t="s">
+        <v>23</v>
+      </c>
+      <c r="D57" t="s">
+        <v>26</v>
+      </c>
+      <c r="E57">
+        <v>1.781530065237729</v>
+      </c>
+      <c r="F57">
+        <v>0.5075966032810001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58">
+        <v>9</v>
+      </c>
+      <c r="B58" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" t="s">
+        <v>23</v>
+      </c>
+      <c r="D58" t="s">
+        <v>27</v>
+      </c>
+      <c r="E58">
+        <v>0.5785160493039088</v>
+      </c>
+      <c r="F58">
+        <v>0.5075966032810001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59">
+        <v>9</v>
+      </c>
+      <c r="B59" t="s">
+        <v>12</v>
+      </c>
+      <c r="C59" t="s">
+        <v>23</v>
+      </c>
+      <c r="D59" t="s">
+        <v>31</v>
+      </c>
+      <c r="E59">
+        <v>43.14002190292393</v>
+      </c>
+      <c r="F59">
+        <v>0.5075966032810001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60">
+        <v>9</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" t="s">
+        <v>23</v>
+      </c>
+      <c r="D60" t="s">
+        <v>28</v>
+      </c>
+      <c r="E60">
+        <v>1109719.797519233</v>
+      </c>
+      <c r="F60">
+        <v>0.5075966032810001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61">
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
+        <v>11</v>
+      </c>
+      <c r="C61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D61" t="s">
+        <v>29</v>
+      </c>
+      <c r="E61">
+        <v>1.88536087034721</v>
+      </c>
+      <c r="F61">
+        <v>0.5076115735595489</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62">
+        <v>10</v>
+      </c>
+      <c r="B62" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" t="s">
+        <v>23</v>
+      </c>
+      <c r="D62" t="s">
+        <v>26</v>
+      </c>
+      <c r="E62">
+        <v>1.781530065237729</v>
+      </c>
+      <c r="F62">
+        <v>0.5076115735595489</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63">
+        <v>10</v>
+      </c>
+      <c r="B63" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" t="s">
+        <v>23</v>
+      </c>
+      <c r="D63" t="s">
+        <v>27</v>
+      </c>
+      <c r="E63">
+        <v>0.3680594446428271</v>
+      </c>
+      <c r="F63">
+        <v>0.5076115735595489</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64">
+        <v>10</v>
+      </c>
+      <c r="B64" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" t="s">
+        <v>23</v>
+      </c>
+      <c r="D64" t="s">
+        <v>31</v>
+      </c>
+      <c r="E64">
+        <v>78.15608186298728</v>
+      </c>
+      <c r="F64">
+        <v>0.5076115735595489</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65">
+        <v>10</v>
+      </c>
+      <c r="B65" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" t="s">
+        <v>23</v>
+      </c>
+      <c r="D65" t="s">
+        <v>28</v>
+      </c>
+      <c r="E65">
+        <v>1442095.15756404</v>
+      </c>
+      <c r="F65">
+        <v>0.5076115735595489</v>
       </c>
     </row>
   </sheetData>
@@ -1189,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1197,10 +1851,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1208,10 +1862,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>652.1993414109966</v>
+        <v>663.756448493994</v>
       </c>
       <c r="C2">
-        <v>0.1811664837252768</v>
+        <v>0.1843767912483316</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1219,10 +1873,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>624.6746508350006</v>
+        <v>663.7742048969958</v>
       </c>
       <c r="C3">
-        <v>0.1735207363430557</v>
+        <v>0.1843817235824988</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1230,10 +1884,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>630.1063828060032</v>
+        <v>657.2089480600116</v>
       </c>
       <c r="C4">
-        <v>0.1750295507794453</v>
+        <v>0.182558041127781</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1241,10 +1895,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>640.7010529990002</v>
+        <v>648.7044128569978</v>
       </c>
       <c r="C5">
-        <v>0.1779725147219445</v>
+        <v>0.1801956702380549</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1252,10 +1906,65 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>628.2668139600028</v>
+        <v>642.2604205889947</v>
       </c>
       <c r="C6">
-        <v>0.1745185594333341</v>
+        <v>0.1784056723858319</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>3942.215850574998</v>
+      </c>
+      <c r="C7">
+        <v>1.095059958493055</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>625.7405641259975</v>
+      </c>
+      <c r="C8">
+        <v>0.1738168233683326</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>5214.774633763998</v>
+      </c>
+      <c r="C9">
+        <v>1.448548509378888</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>623.7839413000038</v>
+      </c>
+      <c r="C10">
+        <v>0.1732733170277788</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>653.4349003530078</v>
+      </c>
+      <c r="C11">
+        <v>0.1815096945425022</v>
       </c>
     </row>
   </sheetData>
@@ -1265,7 +1974,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1273,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1281,7 +1990,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.2932606537898456</v>
+        <v>0.4934549302530007</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1289,7 +1998,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.2992443668463679</v>
+        <v>0.5053434469268637</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1297,7 +2006,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.2992564839485203</v>
+        <v>0.5054794068756243</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1305,7 +2014,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.2992564839485203</v>
+        <v>0.5055339631996827</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1313,7 +2022,47 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.2992566480378244</v>
+        <v>0.5057333829338057</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0.5057930987636794</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>0.5058249729715975</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0.5073603959468733</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>0.5075966491921295</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0.5076116194706783</v>
       </c>
     </row>
   </sheetData>
@@ -1328,18 +2077,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="B2">
         <v>-0.002944</v>
@@ -1350,7 +2099,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="B3">
         <v>-0.004340256958025938</v>
@@ -1361,7 +2110,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="B4">
         <v>-0.004340256958025938</v>
@@ -1372,7 +2121,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B5">
         <v>-0.004340256958025938</v>
@@ -1383,7 +2132,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B6">
         <v>-0.004340256958025938</v>

</xml_diff>